<commit_message>
feat(etf): log-return option + daily return-analysis workflow
- etf_returns.py: add a `method` param ('simple' default | 'log') threaded
  through period_return/compute_returns/reports and a `--method` CLI flag.
  Log returns are ln(close/base); both conventions preserve ranking order, so
  top/bottom lists are identical and only magnitudes change. Report headers now
  state the convention. (TDD: log value + invalid-method guard.)
- .github/workflows/etf_returns.yml: run the analysis after each "Download
  Daily OHLC Data" completes (workflow_run) + workflow_dispatch, committing the
  three report files with [skip ci] and a rebase-retry push. Pure pandas over
  the committed parquet — no network / algoshort.

54 ETF tests green.
</commit_message>
<xml_diff>
--- a/data/results/etf/returns_ranking.xlsx
+++ b/data/results/etf/returns_ranking.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -586,6 +586,81 @@
       <c r="C11" t="inlineStr">
         <is>
           <t>Amundi EURO STOXX 50 Daily (-2x) Inverse UCITS ETF Acc</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>BCCMA.SW</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0.03691437376361972</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>UBS BBG Commodity CMCI SF UCITS ETF USD acc</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>TELE.PA</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0.03452904661767775</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Amundi STOXX Europe 600 Telecommunications UCITS ETF Acc</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>ABBA.SW</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>0.02807797708419013</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>21shares Bitcoin Ethereum Core ETP</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>FBTC.MI</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>0.02677895973065669</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Fidelity Physical Bitcoin ETP</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>INDO.PA</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>0.02462910956296205</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Amundi MSCI Indonesia UCITS ETF Acc</t>
         </is>
       </c>
     </row>
@@ -600,7 +675,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -767,6 +842,81 @@
       <c r="C11" t="inlineStr">
         <is>
           <t>BNP Paribas Easy ESG Enhanced US UCITS ETF EUR Hedged Acc</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>FBT.MI</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0.1045520414775176</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>First Trust NYSE Arca Biotechnology UCITS ETF Acc</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>BTEC.SW</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0.08783161148811036</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>iShares Nasdaq US Biotechnology UCITS ETF</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>BSOL.PA</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>0.08534640049685427</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Bitwise Solana Staking ETP</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>ARKK.MI</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>0.07998883393049838</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>ARK Innovation UCITS ETF USD Accumulating</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>SETH.AS</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>0.07784429950385774</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>AMINA Ethereum ETP</t>
         </is>
       </c>
     </row>
@@ -781,7 +931,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -948,6 +1098,81 @@
       <c r="C11" t="inlineStr">
         <is>
           <t>Amundi MSCI Korea UCITS ETF Acc</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>IKRA.AS</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0.2685487917573555</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>iShares MSCI Korea UCITS ETF (Dist)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>GOAI.AS</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0.2558051926830418</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Amundi MSCI Robotics &amp; AI UCITS ETF Acc</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>FBT.MI</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>0.2375407799057305</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>First Trust NYSE Arca Biotechnology UCITS ETF Acc</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>WITS.AS</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>0.2352438044925331</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>iShares MSCI World Information Technology Sector Advanced UCITS ETF USD (Dist)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>GLIT.PA</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>0.232112574980101</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Amundi S&amp;P Global Information Technology ESG UCITS ETF DR EUR (A)</t>
         </is>
       </c>
     </row>
@@ -962,7 +1187,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1129,6 +1354,81 @@
       <c r="C11" t="inlineStr">
         <is>
           <t>Amundi Core S&amp;P 500 Swap UCITS ETF Acc</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>NRGW.PA</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0.2642900387483433</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Amundi S&amp;P Global Energy Carbon Reduced UCITS ETF DR EUR (A)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>EXCD.AS</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0.2564886970946796</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>iShares MSCI EM ex-China UCITS ETF USD (Dist)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>SXLE.AS</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>0.2498896474626309</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>State Street SPDR S&amp;P U.S. Energy Select Sector UCITS ETF USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>FTAI.MI</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>0.2482117355335969</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>First Trust Bloomberg Artificial Intelligence UCITS ETF Class A Accumulation</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>FEME.MI</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>0.245093498057402</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Fidelity Emerging Markets Quality Income UCITS ETF INC-USD</t>
         </is>
       </c>
     </row>
@@ -1143,7 +1443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1310,6 +1610,81 @@
       <c r="C11" t="inlineStr">
         <is>
           <t>Vanguard FTSE Developed Asia Pacific ex Japan UCITS ETF (USD) Accumulating</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>EMXC.PA</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0.5742624509571184</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Amundi MSCI Emerging Ex China UCITS ETF Acc</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>BRES.PA</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0.5643582343116078</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Amundi STOXX Europe 600 Basic Resources UCITS ETF Acc</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>TPHG.PA</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>0.5324881080680428</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Amundi Japan Topix UCITS ETF Daily Hedged GBP</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>BNK.PA</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>0.5322475923100316</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Amundi STOXX Europe 600 Banks UCITS ETF Acc</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>EXCD.AS</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>0.5299646630586388</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>iShares MSCI EM ex-China UCITS ETF USD (Dist)</t>
         </is>
       </c>
     </row>
@@ -1324,7 +1699,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1491,6 +1866,81 @@
       <c r="C11" t="inlineStr">
         <is>
           <t>Amundi Japan Topix UCITS ETF Daily Hedged USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>GRE.PA</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>1.157711829953367</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Amundi MSCI Greece UCITS ETF Dist</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>JPHU.PA</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>1.153712096333823</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Amundi JPX Nikkei 400 UCITS ETF Daily Hedged USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>JPHG.PA</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>1.130249633900089</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Amundi JPX Nikkei 400 UCITS ETF Daily Hedged GBP</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>TPHG.PA</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>1.123865672814606</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Amundi Japan Topix UCITS ETF Daily Hedged GBP</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>MIB.PA</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>1.106605816728025</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Amundi FTSE MIB UCITS ETF Dist</t>
         </is>
       </c>
     </row>
@@ -1505,7 +1955,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1675,6 +2125,81 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>SXLE.AS</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0.2957373514562294</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>State Street SPDR S&amp;P U.S. Energy Select Sector UCITS ETF USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>FEMI.MI</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0.294412338744366</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Fidelity Emerging Markets Quality Income UCITS ETF ACC-USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>NRGW.PA</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>0.2908254029383845</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Amundi S&amp;P Global Energy Carbon Reduced UCITS ETF DR EUR (A)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>SP5C.PA</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>0.2888175993127151</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Amundi Core S&amp;P 500 Swap UCITS ETF Acc</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>STN.PA</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>0.2870218647235494</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>State Street SPDR MSCI Europe Energy UCITS ETF EUR</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(etf): illiquidity screen for the return analysis
Thin ETFs (obscure crypto ETPs, tiny listings) with stale/erratic prints were
dominating the return boards. Add a liquidity screen applied before ranking.

- etf_liquidity.py: liquidity_stats (median daily traded value = close*volume,
  and active-days fraction over a lookback) + liquid_symbols (both floors).
- etf_returns.py: filter the universe to liquid symbols before ranking, with
  --min-traded-value / --min-active / --liquidity-lookback / --no-liquidity-filter
  and a screen note in the report headers. Defaults: >= 50,000 median daily
  traded value & >= 80% active days over 90d (keeps ~252 of ~554).

Result: the thin crypto ETPs (TIAB/AUNI/ET32...) drop out; real liquid movers
remain. Orthogonal to the LQQ.PA/JPXX.L split/re-denomination data artifacts
(those are liquid — a separate sanity check). TDD'd; 15 return/liquidity tests.
</commit_message>
<xml_diff>
--- a/data/results/etf/returns_ranking.xlsx
+++ b/data/results/etf/returns_ranking.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -442,225 +442,120 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>TIAB.PA</t>
+          <t>STN.PA</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.1244270225218909</v>
+        <v>0.07088469158115274</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Bitwise Celestia Staking ETP</t>
+          <t>State Street SPDR MSCI Europe Energy UCITS ETF EUR</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>AUNI.AS</t>
+          <t>DSD.PA</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.1234758013921327</v>
+        <v>0.05913640588672275</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>21shares Uniswap ETP</t>
+          <t>Amundi ShortDAX Daily (-2x) Inverse UCITS ETF Acc</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ET32.PA</t>
+          <t>SXLE.AS</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.08659070370634114</v>
+        <v>0.05750153606847408</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Bitwise Ethereum Staking ETP</t>
+          <t>State Street SPDR S&amp;P U.S. Energy Select Sector UCITS ETF USD</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>STN.PA</t>
+          <t>NRGW.PA</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.07088469158115274</v>
+        <v>0.0489349675918187</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>State Street SPDR MSCI Europe Energy UCITS ETF EUR</t>
+          <t>Amundi S&amp;P Global Energy Carbon Reduced UCITS ETF DR EUR (A)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>SDOT.AS</t>
+          <t>BXX.PA</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.06692913047073046</v>
+        <v>0.04206313555654373</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>AMINA Polkadot ETP</t>
+          <t>Amundi EURO STOXX 50 Daily (-2x) Inverse UCITS ETF Acc</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ADOT.AS</t>
+          <t>TELE.PA</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.06675130324650169</v>
+        <v>0.03452904661767775</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>21shares Polkadot ETP</t>
+          <t>Amundi STOXX Europe 600 Telecommunications UCITS ETF Acc</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>DSD.PA</t>
+          <t>INDO.PA</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.05913640588672275</v>
+        <v>0.02462910956296205</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Amundi ShortDAX Daily (-2x) Inverse UCITS ETF Acc</t>
+          <t>Amundi MSCI Indonesia UCITS ETF Acc</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>SXLE.AS</t>
+          <t>BSX.PA</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.05750153606847408</v>
+        <v>0.02166618866541903</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>State Street SPDR S&amp;P U.S. Energy Select Sector UCITS ETF USD</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>NRGW.PA</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>0.0489349675918187</v>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Amundi S&amp;P Global Energy Carbon Reduced UCITS ETF DR EUR (A)</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>BXX.PA</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>0.04206313555654373</v>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Amundi EURO STOXX 50 Daily (-2x) Inverse UCITS ETF Acc</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>BCCMA.SW</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>0.03691437376361972</v>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>UBS BBG Commodity CMCI SF UCITS ETF USD acc</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>TELE.PA</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>0.03452904661767775</v>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Amundi STOXX Europe 600 Telecommunications UCITS ETF Acc</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>ABBA.SW</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>0.02807797708419013</v>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>21shares Bitcoin Ethereum Core ETP</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>FBTC.MI</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>0.02677895973065669</v>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Fidelity Physical Bitcoin ETP</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>INDO.PA</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>0.02462910956296205</v>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Amundi MSCI Indonesia UCITS ETF Acc</t>
+          <t>Amundi EURO STOXX 50 Daily (-1x) Inverse UCITS ETF Acc</t>
         </is>
       </c>
     </row>
@@ -675,7 +570,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -698,225 +593,120 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>AUNI.AS</t>
+          <t>ARKG.MI</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.4497998976697066</v>
+        <v>0.2302223837755073</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>21shares Uniswap ETP</t>
+          <t>ARK Genomic Revolution UCITS ETF USD Accumulating</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>TIAB.PA</t>
+          <t>SP5C.PA</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.3909591383710396</v>
+        <v>0.1703637705238301</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Bitwise Celestia Staking ETP</t>
+          <t>Amundi Core S&amp;P 500 Swap UCITS ETF Acc</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ARKG.MI</t>
+          <t>BTEC.SW</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.2302223837755073</v>
+        <v>0.08783161148811036</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>ARK Genomic Revolution UCITS ETF USD Accumulating</t>
+          <t>iShares Nasdaq US Biotechnology UCITS ETF</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>JSOL.AS</t>
+          <t>ARKK.MI</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.1841651948457452</v>
+        <v>0.07998883393049838</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>21shares Jito Staked SOL ETP</t>
+          <t>ARK Innovation UCITS ETF USD Accumulating</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CSOL.MI</t>
+          <t>BNKE.PA</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.175791442448135</v>
+        <v>0.07761454350890928</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>21shares Solana Core Staking ETP</t>
+          <t>Amundi Euro Stoxx Banks UCITS ETF Acc</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>SP5C.PA</t>
+          <t>STZ.PA</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.1703637705238301</v>
+        <v>0.07619972786979612</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Amundi Core S&amp;P 500 Swap UCITS ETF Acc</t>
+          <t>State Street SPDR MSCI Europe Financials UCITS ETF EUR</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ASOL.AS</t>
+          <t>BNK.PA</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.1492440483785455</v>
+        <v>0.07408527478270366</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>21shares Solana Staking ETP</t>
+          <t>Amundi STOXX Europe 600 Banks UCITS ETF Acc</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>QUSAE.PA</t>
+          <t>XDWF.MI</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.1397838360603161</v>
+        <v>0.06616888992604664</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy Alpha Enhanced US UCITS ETF EUR Acc</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>SLNC.PA</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>0.1377138068537653</v>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>CoinShares Physical Staked Solana</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>AUSSH.PA</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>0.1307394352806199</v>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>BNP Paribas Easy ESG Enhanced US UCITS ETF EUR Hedged Acc</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>FBT.MI</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>0.1045520414775176</v>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>First Trust NYSE Arca Biotechnology UCITS ETF Acc</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>BTEC.SW</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>0.08783161148811036</v>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>iShares Nasdaq US Biotechnology UCITS ETF</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>BSOL.PA</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>0.08534640049685427</v>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Bitwise Solana Staking ETP</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>ARKK.MI</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>0.07998883393049838</v>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>ARK Innovation UCITS ETF USD Accumulating</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>SETH.AS</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>0.07784429950385774</v>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>AMINA Ethereum ETP</t>
+          <t>Xtrackers MSCI World Financials UCITS ETF 1C</t>
         </is>
       </c>
     </row>
@@ -931,7 +721,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -984,195 +774,90 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>NEAR.AS</t>
+          <t>SP5C.PA</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.368990242986162</v>
+        <v>0.2932447794350908</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>21shares NEAR Protocol Staking ETP</t>
+          <t>Amundi Core S&amp;P 500 Swap UCITS ETF Acc</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>EJAPU.PA</t>
+          <t>CL2.PA</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.3451283397940894</v>
+        <v>0.2878198938069461</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy MSCI Japan Min TE UCITS ETF USD</t>
+          <t>Amundi MSCI USA Daily (2x) Leveraged UCITS ETF Acc</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ONDO.AS</t>
+          <t>LEVMIB.MI</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.324706994489665</v>
+        <v>0.2686936913329221</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>21Shares Ondo ETP</t>
+          <t>Amundi FTSE MIB Daily (2x) Leveraged UCITS ETF Dist</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>FTAI.MI</t>
+          <t>KRW.PA</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.3104534904029543</v>
+        <v>0.2686860651842049</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>First Trust Bloomberg Artificial Intelligence UCITS ETF Class A Accumulation</t>
+          <t>Amundi MSCI Korea UCITS ETF Acc</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>SP5C.PA</t>
+          <t>IKRA.AS</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.2932447794350908</v>
+        <v>0.2685487917573555</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Amundi Core S&amp;P 500 Swap UCITS ETF Acc</t>
+          <t>iShares MSCI Korea UCITS ETF (Dist)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CL2.PA</t>
+          <t>WITS.AS</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.2878198938069461</v>
+        <v>0.2352438044925331</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Amundi MSCI USA Daily (2x) Leveraged UCITS ETF Acc</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>LEVMIB.MI</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>0.2686936913329221</v>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Amundi FTSE MIB Daily (2x) Leveraged UCITS ETF Dist</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>KRW.PA</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>0.2686860651842049</v>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Amundi MSCI Korea UCITS ETF Acc</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>IKRA.AS</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>0.2685487917573555</v>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>iShares MSCI Korea UCITS ETF (Dist)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>GOAI.AS</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>0.2558051926830418</v>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Amundi MSCI Robotics &amp; AI UCITS ETF Acc</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>FBT.MI</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>0.2375407799057305</v>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>First Trust NYSE Arca Biotechnology UCITS ETF Acc</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>WITS.AS</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>0.2352438044925331</v>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
           <t>iShares MSCI World Information Technology Sector Advanced UCITS ETF USD (Dist)</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>GLIT.PA</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>0.232112574980101</v>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Amundi S&amp;P Global Information Technology ESG UCITS ETF DR EUR (A)</t>
         </is>
       </c>
     </row>
@@ -1187,7 +872,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1270,165 +955,60 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>EJAPU.PA</t>
+          <t>ARKG.MI</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3451283397940894</v>
+        <v>0.3332675507779312</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>BNP Paribas Easy MSCI Japan Min TE UCITS ETF USD</t>
+          <t>ARK Genomic Revolution UCITS ETF USD Accumulating</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ARKG.MI</t>
+          <t>VAPU.SW</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.3332675507779312</v>
+        <v>0.3009325716984608</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ARK Genomic Revolution UCITS ETF USD Accumulating</t>
+          <t>Vanguard FTSE Developed Asia Pacific ex Japan UCITS ETF (USD) Accumulating</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>VAPU.SW</t>
+          <t>STN.PA</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.3009325716984608</v>
+        <v>0.2918728490319493</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Vanguard FTSE Developed Asia Pacific ex Japan UCITS ETF (USD) Accumulating</t>
+          <t>State Street SPDR MSCI Europe Energy UCITS ETF EUR</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>STN.PA</t>
+          <t>EMXC.PA</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.2918728490319493</v>
+        <v>0.2812062625950971</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>State Street SPDR MSCI Europe Energy UCITS ETF EUR</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>EMXC.PA</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>0.2812062625950971</v>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
           <t>Amundi MSCI Emerging Ex China UCITS ETF Acc</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>SP5C.PA</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>0.2656893720769995</v>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Amundi Core S&amp;P 500 Swap UCITS ETF Acc</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>NRGW.PA</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>0.2642900387483433</v>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Amundi S&amp;P Global Energy Carbon Reduced UCITS ETF DR EUR (A)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>EXCD.AS</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>0.2564886970946796</v>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>iShares MSCI EM ex-China UCITS ETF USD (Dist)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>SXLE.AS</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>0.2498896474626309</v>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>State Street SPDR S&amp;P U.S. Energy Select Sector UCITS ETF USD</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>FTAI.MI</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>0.2482117355335969</v>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>First Trust Bloomberg Artificial Intelligence UCITS ETF Class A Accumulation</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>FEME.MI</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>0.245093498057402</v>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Fidelity Emerging Markets Quality Income UCITS ETF INC-USD</t>
         </is>
       </c>
     </row>
@@ -1443,7 +1023,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1496,195 +1076,90 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>MINR.MI</t>
+          <t>AINF.AS</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1.019933503870999</v>
+        <v>0.8904155813543404</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>First Trust Indxx Future Economy Metals UCITS ETF Class A Accumulation</t>
+          <t>iShares AI Infrastructure UCITS ETF USD (Acc)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>AINF.AS</t>
+          <t>LEVMIB.MI</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.8904155813543404</v>
+        <v>0.7765479014724228</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>iShares AI Infrastructure UCITS ETF USD (Acc)</t>
+          <t>Amundi FTSE MIB Daily (2x) Leveraged UCITS ETF Dist</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>LEVMIB.MI</t>
+          <t>COPX.MI</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.7765479014724228</v>
+        <v>0.7714090452057252</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Amundi FTSE MIB Daily (2x) Leveraged UCITS ETF Dist</t>
+          <t>Global X Copper Miners UCITS ETF USD Accumulating</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>COPX.MI</t>
+          <t>BATT.AS</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.7714090452057252</v>
+        <v>0.7222165004178984</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Global X Copper Miners UCITS ETF USD Accumulating</t>
+          <t>L&amp;G Battery Value-Chain UCITS ETF</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>BATT.AS</t>
+          <t>ARKG.MI</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.7222165004178984</v>
+        <v>0.6523443122821793</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>L&amp;G Battery Value-Chain UCITS ETF</t>
+          <t>ARK Genomic Revolution UCITS ETF USD Accumulating</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ARKG.MI</t>
+          <t>VAPU.SW</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.6523443122821793</v>
+        <v>0.5769297947462435</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>ARK Genomic Revolution UCITS ETF USD Accumulating</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>GOAI.AS</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>0.5891469573527659</v>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Amundi MSCI Robotics &amp; AI UCITS ETF Acc</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>VAPU.SW</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>0.5769297947462435</v>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
           <t>Vanguard FTSE Developed Asia Pacific ex Japan UCITS ETF (USD) Accumulating</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>EMXC.PA</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>0.5742624509571184</v>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Amundi MSCI Emerging Ex China UCITS ETF Acc</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>BRES.PA</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>0.5643582343116078</v>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Amundi STOXX Europe 600 Basic Resources UCITS ETF Acc</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>TPHG.PA</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>0.5324881080680428</v>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Amundi Japan Topix UCITS ETF Daily Hedged GBP</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>BNK.PA</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>0.5322475923100316</v>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Amundi STOXX Europe 600 Banks UCITS ETF Acc</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>EXCD.AS</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>0.5299646630586388</v>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>iShares MSCI EM ex-China UCITS ETF USD (Dist)</t>
         </is>
       </c>
     </row>
@@ -1699,7 +1174,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1836,111 +1311,6 @@
       <c r="C9" t="inlineStr">
         <is>
           <t>State Street SPDR MSCI Europe Financials UCITS ETF EUR</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>CEC.PA</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>1.207374345089354</v>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Amundi MSCI Eastern Europe Ex Russia UCITS ETF Acc</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>TPHU.PA</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>1.159602887961937</v>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Amundi Japan Topix UCITS ETF Daily Hedged USD</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>GRE.PA</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>1.157711829953367</v>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Amundi MSCI Greece UCITS ETF Dist</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>JPHU.PA</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>1.153712096333823</v>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Amundi JPX Nikkei 400 UCITS ETF Daily Hedged USD</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>JPHG.PA</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>1.130249633900089</v>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Amundi JPX Nikkei 400 UCITS ETF Daily Hedged GBP</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>TPHG.PA</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>1.123865672814606</v>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Amundi Japan Topix UCITS ETF Daily Hedged GBP</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>MIB.PA</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>1.106605816728025</v>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Amundi FTSE MIB UCITS ETF Dist</t>
         </is>
       </c>
     </row>
@@ -1955,7 +1325,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2095,111 +1465,6 @@
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>EJAPU.PA</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>0.3451283397940894</v>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>BNP Paribas Easy MSCI Japan Min TE UCITS ETF USD</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>FEME.MI</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>0.302805170236357</v>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Fidelity Emerging Markets Quality Income UCITS ETF INC-USD</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>SXLE.AS</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>0.2957373514562294</v>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>State Street SPDR S&amp;P U.S. Energy Select Sector UCITS ETF USD</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>FEMI.MI</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>0.294412338744366</v>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Fidelity Emerging Markets Quality Income UCITS ETF ACC-USD</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>NRGW.PA</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>0.2908254029383845</v>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Amundi S&amp;P Global Energy Carbon Reduced UCITS ETF DR EUR (A)</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>SP5C.PA</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>0.2888175993127151</v>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Amundi Core S&amp;P 500 Swap UCITS ETF Acc</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>STN.PA</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>0.2870218647235494</v>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>State Street SPDR MSCI Europe Energy UCITS ETF EUR</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>